<commit_message>
[Data] 변경된 Data Table 임시 적용 - Player Move, Enemy State
테스트를 위해 커밋
추가 적용 필요
</commit_message>
<xml_diff>
--- a/Assets/06 Data/ExcelData/dt_player_move_stats.xlsx
+++ b/Assets/06 Data/ExcelData/dt_player_move_stats.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\덕코프 기획\데이터테이블\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StudyUnity\Duckov\Assets\06 Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E488EE-E0A8-4EBF-9CB4-6AD3CE9ACACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FC0FC4-131B-4640-8FC8-637C33AE82D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9690" yWindow="3765" windowWidth="18225" windowHeight="7140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -665,7 +665,7 @@
         <v>1.5</v>
       </c>
       <c r="G4" s="6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H4" s="5">
         <v>0.5</v>

</xml_diff>

<commit_message>
[Chore] 구르기 거리 적용(PlayerMoveStatsData) 및 이동거리 증가
</commit_message>
<xml_diff>
--- a/Assets/06 Data/ExcelData/dt_player_move_stats.xlsx
+++ b/Assets/06 Data/ExcelData/dt_player_move_stats.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Genie\Desktop\duckov-clone\Assets\06 Data\ExcelData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StudyUnity\Duckov\Assets\06 Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{145CB48B-17EF-4C0D-A415-1C2AB196C796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FABDE8-6C66-48DF-8ADF-E48FD8D4CEB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5325" yWindow="4185" windowWidth="20595" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7665" yWindow="2895" windowWidth="20190" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -665,19 +665,19 @@
         <v>1.5</v>
       </c>
       <c r="G4" s="6">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H4" s="5">
         <v>0.5</v>
       </c>
       <c r="I4" s="5">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="J4" s="6">
         <v>10</v>
       </c>
       <c r="K4" s="5">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>